<commit_message>
Owner's browser check passed: report and README updated
The footer Admin link, thank-you heading, typed guest count and price entry
after the lint fix were tested in the browser by the owner; all work.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reports/StepIn-Development-Test-Report-2026-10-20.xlsx
+++ b/Reports/StepIn-Development-Test-Report-2026-10-20.xlsx
@@ -1677,7 +1677,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Typecheck clean. Not clicked through in a browser (the dev server was stopped for low memory).</t>
+          <t>Pass: typecheck clean; tested in the browser by the owner.</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -2119,32 +2119,32 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Changes not yet seen in a browser</t>
+          <t>Browser check by the owner</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Footer Admin link, "Thank you for Stepping In :-)" heading, typed guest count, euro field after the lint change.</t>
+          <t>Footer Admin link, "Thank you for Stepping In :-)" heading, typed guest count, entering a price in the admin after the lint change.</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Not run: the dev server was stopped by Claude Code for low memory and not restarted.</t>
+          <t>Pass: the owner tested each one in the browser; all work.</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Typecheck and automated tests only; the e2e homepage test now checks the footer Admin link but was not run.</t>
+          <t>None needed.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="H37" s="9" t="inlineStr">
-        <is>
-          <t>Not tested</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>

</xml_diff>